<commit_message>
Audit complet: correctif F1 (total facture multi-lignes via SUMIFS) + rapport 07_audit_complet
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KLPjvBwSxieSwYM5jVrsXK
</commit_message>
<xml_diff>
--- a/output/ORA_ORA_SSR_v0.xlsx
+++ b/output/ORA_ORA_SSR_v0.xlsx
@@ -52403,7 +52403,7 @@
     <row r="18" ht="16" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>Tarif unitaire :</t>
+          <t>Tarif unitaire (1re ligne) :</t>
         </is>
       </c>
       <c r="B18" s="11">
@@ -52414,11 +52414,11 @@
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>Nb de journées :</t>
+          <t>Nb de journées (total facture) :</t>
         </is>
       </c>
       <c r="B19" s="12">
-        <f>_xlfn.XLOOKUP($B$3,tSuiviFactures[N_DE_FACTURE],tSuiviFactures[Nb_journees],0)</f>
+        <f>SUMIFS(tSuiviFactures[Nb_journees],tSuiviFactures[N_DE_FACTURE],$B$3)</f>
         <v/>
       </c>
     </row>
@@ -52430,7 +52430,7 @@
         </is>
       </c>
       <c r="B21" s="13">
-        <f>IF(OR(B18="",B19=""),"",B18*B19)</f>
+        <f>IF($B$3="","",SUMIFS(tSuiviFactures[Montant],tSuiviFactures[N_DE_FACTURE],$B$3))</f>
         <v/>
       </c>
     </row>

</xml_diff>